<commit_message>
Add migration phases, projections, and throughput capacity to spreadsheet
Extend Actual vs Planned XLSX with Migration Phases (900/8024/14000 min
processing times), Phase Timeline milestones, and Projections sheet with
estimated finish dates for 8.5K, 11.5K, and full 35K account goals.

Co-authored-by: maiagordon-commits <maiagordon-commits@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/migration_actual_vs_planned.xlsx
+++ b/migration_actual_vs_planned.xlsx
@@ -9,14 +9,17 @@
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
     <sheet name="Weekly Detail" sheetId="2" r:id="rId2"/>
-    <sheet name="Chart" sheetId="3" r:id="rId3"/>
+    <sheet name="Migration Phases" sheetId="3" r:id="rId3"/>
+    <sheet name="Phase Timeline" sheetId="4" r:id="rId4"/>
+    <sheet name="Projections" sheetId="5" r:id="rId5"/>
+    <sheet name="Chart" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="88">
   <si>
     <t>Week Starting</t>
   </si>
@@ -84,7 +87,202 @@
     <t>Weekly Total</t>
   </si>
   <si>
-    <t>To use in Google Sheets: Upload this file to Google Drive → Open with Google Sheets. Edit values on the Data tab; recreate the chart via Insert → Chart if needed.</t>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Days</t>
+  </si>
+  <si>
+    <t>Avg Res/Day</t>
+  </si>
+  <si>
+    <t>Total Reservations</t>
+  </si>
+  <si>
+    <t>Accounts (Phase)</t>
+  </si>
+  <si>
+    <t>Avg Res/Account</t>
+  </si>
+  <si>
+    <t>Processing @ 900/min</t>
+  </si>
+  <si>
+    <t>Processing @ 8,024/min</t>
+  </si>
+  <si>
+    <t>Processing @ 14,000/min</t>
+  </si>
+  <si>
+    <t>Ramp-up</t>
+  </si>
+  <si>
+    <t>8/3/2026</t>
+  </si>
+  <si>
+    <t>2h 38m</t>
+  </si>
+  <si>
+    <t>18m</t>
+  </si>
+  <si>
+    <t>10m</t>
+  </si>
+  <si>
+    <t>Steady Growth</t>
+  </si>
+  <si>
+    <t>8/4/2026</t>
+  </si>
+  <si>
+    <t>9/22/2026</t>
+  </si>
+  <si>
+    <t>4h 12m</t>
+  </si>
+  <si>
+    <t>28m</t>
+  </si>
+  <si>
+    <t>16m</t>
+  </si>
+  <si>
+    <t>Acceleration</t>
+  </si>
+  <si>
+    <t>9/23/2026</t>
+  </si>
+  <si>
+    <t>11/11/2026</t>
+  </si>
+  <si>
+    <t>5h 48m</t>
+  </si>
+  <si>
+    <t>39m</t>
+  </si>
+  <si>
+    <t>22m</t>
+  </si>
+  <si>
+    <t>Full Speed</t>
+  </si>
+  <si>
+    <t>11/12/2026</t>
+  </si>
+  <si>
+    <t>12/31/2026</t>
+  </si>
+  <si>
+    <t>7h 22m</t>
+  </si>
+  <si>
+    <t>50m</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Accounts This Phase</t>
+  </si>
+  <si>
+    <t>Cumulative Accounts</t>
+  </si>
+  <si>
+    <t>Current status (as of 6/15/2026)</t>
+  </si>
+  <si>
+    <t>Recent run rate (accounts/day)</t>
+  </si>
+  <si>
+    <t>Goal</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Accounts/Day</t>
+  </si>
+  <si>
+    <t>Days Remaining</t>
+  </si>
+  <si>
+    <t>Projected Finish</t>
+  </si>
+  <si>
+    <t>Planned Finish</t>
+  </si>
+  <si>
+    <t>Days Ahead of Plan</t>
+  </si>
+  <si>
+    <t>Near-term goal (8,500 accounts)</t>
+  </si>
+  <si>
+    <t>Current pace</t>
+  </si>
+  <si>
+    <t>07/02/2026</t>
+  </si>
+  <si>
+    <t>7/13/2026</t>
+  </si>
+  <si>
+    <t>Ramp-up phase pace</t>
+  </si>
+  <si>
+    <t>07/06/2026</t>
+  </si>
+  <si>
+    <t>Near-term plan pace</t>
+  </si>
+  <si>
+    <t>07/16/2026</t>
+  </si>
+  <si>
+    <t>End of Ramp-up (11,509 accounts)</t>
+  </si>
+  <si>
+    <t>07/13/2026</t>
+  </si>
+  <si>
+    <t>07/19/2026</t>
+  </si>
+  <si>
+    <t>08/03/2026</t>
+  </si>
+  <si>
+    <t>Full program (~35,001 accounts)</t>
+  </si>
+  <si>
+    <t>10/06/2026</t>
+  </si>
+  <si>
+    <t>10/29/2026</t>
+  </si>
+  <si>
+    <t>12/29/2026</t>
+  </si>
+  <si>
+    <t>Days Ahead of Plan = positive means finishing BEFORE planned date. Based on 3,576 accounts as of 6/15/2026.</t>
+  </si>
+  <si>
+    <t>Note: Full program projection assumes constant account pace. Later phases (Steady Growth → Full Speed) require 2–4× more reservations per account; reservation throughput (900 vs 8,024 vs 14,000/min) may constrain finish date even if account onboarding stays ahead.</t>
+  </si>
+  <si>
+    <t>To use in Google Sheets: Upload to Google Drive → Open with Google Sheets. Edit Data / Migration Phases / Projections tabs. Tabs: Data, Weekly Detail, Migration Phases, Phase Timeline, Projections, Chart.</t>
   </si>
 </sst>
 </file>
@@ -95,7 +293,7 @@
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="+#,##0;-#,##0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,6 +305,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF2E9E5B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -161,7 +366,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -169,7 +374,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1251,12 +1457,604 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="5" max="8" width="16.7109375" customWidth="1"/>
+    <col min="9" max="11" width="14.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="3">
+        <v>50</v>
+      </c>
+      <c r="E2" s="3">
+        <v>142000</v>
+      </c>
+      <c r="F2" s="3">
+        <v>7090000</v>
+      </c>
+      <c r="G2" s="3">
+        <v>11509</v>
+      </c>
+      <c r="H2" s="3">
+        <v>616</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="3">
+        <v>50</v>
+      </c>
+      <c r="E3" s="3">
+        <v>227200</v>
+      </c>
+      <c r="F3" s="3">
+        <v>11360000</v>
+      </c>
+      <c r="G3" s="3">
+        <v>8513</v>
+      </c>
+      <c r="H3" s="3">
+        <v>1335</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3">
+        <v>50</v>
+      </c>
+      <c r="E4" s="3">
+        <v>312800</v>
+      </c>
+      <c r="F4" s="3">
+        <v>15640000</v>
+      </c>
+      <c r="G4" s="3">
+        <v>7689</v>
+      </c>
+      <c r="H4" s="3">
+        <v>2034</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="3">
+        <v>50</v>
+      </c>
+      <c r="E5" s="3">
+        <v>398200</v>
+      </c>
+      <c r="F5" s="3">
+        <v>19910000</v>
+      </c>
+      <c r="G5" s="3">
+        <v>7290</v>
+      </c>
+      <c r="H5" s="3">
+        <v>2731</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="3">
+        <v>200</v>
+      </c>
+      <c r="F6" s="3">
+        <v>54000000</v>
+      </c>
+      <c r="G6" s="3">
+        <v>35001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="4" width="22.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="3">
+        <v>11509</v>
+      </c>
+      <c r="D2" s="3">
+        <v>11509</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="3">
+        <v>8513</v>
+      </c>
+      <c r="D3" s="3">
+        <v>20022</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="3">
+        <v>7689</v>
+      </c>
+      <c r="D4" s="3">
+        <v>27711</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="3">
+        <v>7290</v>
+      </c>
+      <c r="D5" s="3">
+        <v>35001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="3">
+        <v>3576</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="3">
+        <v>277.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="2" max="8" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="3">
+        <v>8500</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" s="3">
+        <v>277.7</v>
+      </c>
+      <c r="E2" s="3">
+        <v>17.7</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H2" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="3">
+        <v>8500</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="3">
+        <v>230.2</v>
+      </c>
+      <c r="E3" s="3">
+        <v>21.4</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H3" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="3">
+        <v>8500</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="3">
+        <v>158.8</v>
+      </c>
+      <c r="E4" s="3">
+        <v>31</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="4">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="3">
+        <v>11509</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="3">
+        <v>277.7</v>
+      </c>
+      <c r="E5" s="3">
+        <v>28.6</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="3">
+        <v>11509</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="3">
+        <v>230.2</v>
+      </c>
+      <c r="E6" s="3">
+        <v>34.5</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="3">
+        <v>11509</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="3">
+        <v>158.8</v>
+      </c>
+      <c r="E7" s="3">
+        <v>49.9</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="3">
+        <v>35001</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="3">
+        <v>277.7</v>
+      </c>
+      <c r="E8" s="3">
+        <v>113.2</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="5">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="3">
+        <v>35001</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="3">
+        <v>230.2</v>
+      </c>
+      <c r="E9" s="3">
+        <v>136.5</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" s="5">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="3">
+        <v>35001</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="3">
+        <v>158.8</v>
+      </c>
+      <c r="E10" s="3">
+        <v>197.8</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="28" spans="2:2">
-      <c r="B28" s="5" t="s">
-        <v>22</v>
+      <c r="B28" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix cumulative totals: use weekly increments through 6/22
Correct 6/15 and add 6/22 weekly data from latest sheet. Each row is
weekly-only; Cumulative Total column sums all prior weeks. 6/22 total is
2,493 (779 lite + 1,705 pro + 9 enterprise).

Co-authored-by: maiagordon-commits <maiagordon-commits@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/migration_actual_vs_planned.xlsx
+++ b/migration_actual_vs_planned.xlsx
@@ -19,21 +19,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="93">
   <si>
     <t>Week Starting</t>
   </si>
   <si>
-    <t>Weekly Actual</t>
-  </si>
-  <si>
-    <t>Cumulative Actual</t>
+    <t>Weekly Lite</t>
+  </si>
+  <si>
+    <t>Weekly Pro</t>
+  </si>
+  <si>
+    <t>Weekly Enterprise</t>
+  </si>
+  <si>
+    <t>Weekly Total</t>
+  </si>
+  <si>
+    <t>Cumulative Lite</t>
+  </si>
+  <si>
+    <t>Cumulative Pro</t>
+  </si>
+  <si>
+    <t>Cumulative Enterprise</t>
+  </si>
+  <si>
+    <t>Cumulative Total</t>
   </si>
   <si>
     <t>Planned Cumulative</t>
   </si>
   <si>
-    <t>Variance (Actual - Planned)</t>
+    <t>Variance</t>
   </si>
   <si>
     <t>4/13/2026</t>
@@ -84,9 +102,6 @@
     <t>Enterprise</t>
   </si>
   <si>
-    <t>Weekly Total</t>
-  </si>
-  <si>
     <t>Phase</t>
   </si>
   <si>
@@ -198,7 +213,7 @@
     <t>Cumulative Accounts</t>
   </si>
   <si>
-    <t>Current status (as of 6/15/2026)</t>
+    <t>Current status (as of 6/22/2026)</t>
   </si>
   <si>
     <t>Recent run rate (accounts/day)</t>
@@ -234,7 +249,7 @@
     <t>Current pace</t>
   </si>
   <si>
-    <t>07/02/2026</t>
+    <t>09/06/2026</t>
   </si>
   <si>
     <t>7/13/2026</t>
@@ -243,40 +258,40 @@
     <t>Ramp-up phase pace</t>
   </si>
   <si>
-    <t>07/06/2026</t>
+    <t>07/18/2026</t>
   </si>
   <si>
     <t>Near-term plan pace</t>
   </si>
   <si>
-    <t>07/16/2026</t>
+    <t>07/23/2026</t>
   </si>
   <si>
     <t>End of Ramp-up (11,509 accounts)</t>
   </si>
   <si>
-    <t>07/13/2026</t>
-  </si>
-  <si>
-    <t>07/19/2026</t>
-  </si>
-  <si>
-    <t>08/03/2026</t>
+    <t>10/15/2026</t>
+  </si>
+  <si>
+    <t>07/31/2026</t>
+  </si>
+  <si>
+    <t>08/07/2026</t>
   </si>
   <si>
     <t>Full program (~35,001 accounts)</t>
   </si>
   <si>
-    <t>10/06/2026</t>
-  </si>
-  <si>
-    <t>10/29/2026</t>
-  </si>
-  <si>
-    <t>12/29/2026</t>
-  </si>
-  <si>
-    <t>Days Ahead of Plan = positive means finishing BEFORE planned date. Based on 3,576 accounts as of 6/15/2026.</t>
+    <t>08/10/2027</t>
+  </si>
+  <si>
+    <t>11/10/2026</t>
+  </si>
+  <si>
+    <t>12/06/2026</t>
+  </si>
+  <si>
+    <t>Days Ahead of Plan = positive means finishing BEFORE planned date. Based on 2,493 accounts as of 6/22/2026.</t>
   </si>
   <si>
     <t>Note: Full program projection assumes constant account pace. Later phases (Steady Growth → Full Speed) require 2–4× more reservations per account; reservation throughput (900 vs 8,024 vs 14,000/min) may constrain finish date even if account onboarding stays ahead.</t>
@@ -325,7 +340,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -335,6 +350,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1B4F8A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E9E5B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5EE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -366,13 +393,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -484,7 +515,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$14</c:f>
+              <c:f>Data!$I$2:$I$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -516,10 +547,10 @@
                   <c:v>1632</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3576</c:v>
+                  <c:v>1944</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>2493</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -603,7 +634,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$D$2:$D$14</c:f>
+              <c:f>Data!$J$2:$J$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
@@ -1051,14 +1082,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="5" width="18.7109375" customWidth="1"/>
+    <col min="1" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1074,181 +1104,415 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3">
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="4">
         <v>5</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
         <v>5</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="2" t="s">
+      <c r="F2" s="5">
+        <v>5</v>
+      </c>
+      <c r="G2" s="5">
+        <v>0</v>
+      </c>
+      <c r="H2" s="5">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5">
+        <v>5</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4">
+        <v>11</v>
+      </c>
+      <c r="C3" s="4">
+        <v>4</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>15</v>
+      </c>
+      <c r="F3" s="5">
+        <v>16</v>
+      </c>
+      <c r="G3" s="5">
+        <v>4</v>
+      </c>
+      <c r="H3" s="5">
+        <v>0</v>
+      </c>
+      <c r="I3" s="5">
+        <v>20</v>
+      </c>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="4">
+        <v>28</v>
+      </c>
+      <c r="C4" s="4">
+        <v>11</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>39</v>
+      </c>
+      <c r="F4" s="5">
+        <v>44</v>
+      </c>
+      <c r="G4" s="5">
+        <v>15</v>
+      </c>
+      <c r="H4" s="5">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5">
+        <v>59</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="4">
         <v>6</v>
       </c>
-      <c r="B3" s="3">
+      <c r="C5" s="4">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>9</v>
+      </c>
+      <c r="F5" s="5">
+        <v>50</v>
+      </c>
+      <c r="G5" s="5">
+        <v>18</v>
+      </c>
+      <c r="H5" s="5">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5">
+        <v>68</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3">
+      <c r="B6" s="4">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>19</v>
+      </c>
+      <c r="F6" s="5">
+        <v>61</v>
+      </c>
+      <c r="G6" s="5">
+        <v>26</v>
+      </c>
+      <c r="H6" s="5">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5">
+        <v>87</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4">
+        <v>23</v>
+      </c>
+      <c r="C7" s="4">
+        <v>16</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>39</v>
+      </c>
+      <c r="F7" s="5">
+        <v>84</v>
+      </c>
+      <c r="G7" s="5">
+        <v>42</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5">
+        <v>126</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="4">
+        <v>159</v>
+      </c>
+      <c r="C8" s="4">
+        <v>98</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>257</v>
+      </c>
+      <c r="F8" s="5">
+        <v>243</v>
+      </c>
+      <c r="G8" s="5">
+        <v>140</v>
+      </c>
+      <c r="H8" s="5">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5">
+        <v>383</v>
+      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="4">
+        <v>109</v>
+      </c>
+      <c r="C9" s="4">
+        <v>136</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>245</v>
+      </c>
+      <c r="F9" s="5">
+        <v>352</v>
+      </c>
+      <c r="G9" s="5">
+        <v>276</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5">
+        <v>628</v>
+      </c>
+      <c r="J9" s="4">
+        <v>500</v>
+      </c>
+      <c r="K9" s="6">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="4">
+        <v>424</v>
+      </c>
+      <c r="C10" s="4">
+        <v>571</v>
+      </c>
+      <c r="D10" s="4">
+        <v>9</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1004</v>
+      </c>
+      <c r="F10" s="5">
+        <v>776</v>
+      </c>
+      <c r="G10" s="5">
+        <v>847</v>
+      </c>
+      <c r="H10" s="5">
+        <v>9</v>
+      </c>
+      <c r="I10" s="5">
+        <v>1632</v>
+      </c>
+      <c r="J10" s="4">
+        <v>1097</v>
+      </c>
+      <c r="K10" s="6">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3">
-        <v>39</v>
-      </c>
-      <c r="C4" s="3">
-        <v>59</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="3">
+      <c r="B11" s="4">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4">
+        <v>312</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>312</v>
+      </c>
+      <c r="F11" s="5">
+        <v>776</v>
+      </c>
+      <c r="G11" s="5">
+        <v>1159</v>
+      </c>
+      <c r="H11" s="5">
         <v>9</v>
       </c>
-      <c r="C5" s="3">
-        <v>68</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="2" t="s">
+      <c r="I11" s="5">
+        <v>1944</v>
+      </c>
+      <c r="J11" s="4">
+        <v>2650</v>
+      </c>
+      <c r="K11" s="6">
+        <v>-706</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="4">
+        <v>3</v>
+      </c>
+      <c r="C12" s="4">
+        <v>546</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>549</v>
+      </c>
+      <c r="F12" s="5">
+        <v>779</v>
+      </c>
+      <c r="G12" s="5">
+        <v>1705</v>
+      </c>
+      <c r="H12" s="5">
         <v>9</v>
       </c>
-      <c r="B6" s="3">
-        <v>19</v>
-      </c>
-      <c r="C6" s="3">
-        <v>87</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3">
-        <v>39</v>
-      </c>
-      <c r="C7" s="3">
-        <v>126</v>
-      </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="3">
-        <v>257</v>
-      </c>
-      <c r="C8" s="3">
-        <v>383</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="3">
-        <v>245</v>
-      </c>
-      <c r="C9" s="3">
-        <v>628</v>
-      </c>
-      <c r="D9" s="3">
-        <v>500</v>
-      </c>
-      <c r="E9" s="4">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="3">
-        <v>1004</v>
-      </c>
-      <c r="C10" s="3">
-        <v>1632</v>
-      </c>
-      <c r="D10" s="3">
-        <v>1097</v>
-      </c>
-      <c r="E10" s="4">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="3">
-        <v>1944</v>
-      </c>
-      <c r="C11" s="3">
-        <v>3576</v>
-      </c>
-      <c r="D11" s="3">
-        <v>2650</v>
-      </c>
-      <c r="E11" s="4">
-        <v>926</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="3">
+      <c r="I12" s="5">
+        <v>2493</v>
+      </c>
+      <c r="J12" s="4">
         <v>4200</v>
       </c>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="3">
+      <c r="K12" s="6">
+        <v>-1707</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="4">
         <v>5800</v>
       </c>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="3">
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="4">
         <v>7500</v>
       </c>
-      <c r="E14" s="2"/>
+      <c r="K14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1257,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="5" width="14.7109375" customWidth="1"/>
@@ -1268,186 +1532,203 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="4">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4">
+        <v>11</v>
+      </c>
+      <c r="C3" s="4">
+        <v>4</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="4">
+        <v>28</v>
+      </c>
+      <c r="C4" s="4">
+        <v>11</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="4">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="4">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4">
+        <v>23</v>
+      </c>
+      <c r="C7" s="4">
+        <v>16</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="4">
+        <v>159</v>
+      </c>
+      <c r="C8" s="4">
+        <v>98</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B9" s="4">
+        <v>109</v>
+      </c>
+      <c r="C9" s="4">
+        <v>136</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B10" s="4">
+        <v>424</v>
+      </c>
+      <c r="C10" s="4">
+        <v>571</v>
+      </c>
+      <c r="D10" s="4">
+        <v>9</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B11" s="4">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4">
+        <v>312</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3">
-        <v>4</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3">
-        <v>28</v>
-      </c>
-      <c r="C4" s="3">
-        <v>11</v>
-      </c>
-      <c r="D4" s="3">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="3">
-        <v>6</v>
-      </c>
-      <c r="C5" s="3">
+      <c r="B12" s="4">
         <v>3</v>
       </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="3">
-        <v>11</v>
-      </c>
-      <c r="C6" s="3">
-        <v>8</v>
-      </c>
-      <c r="D6" s="3">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3">
-        <v>23</v>
-      </c>
-      <c r="C7" s="3">
-        <v>16</v>
-      </c>
-      <c r="D7" s="3">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="3">
-        <v>159</v>
-      </c>
-      <c r="C8" s="3">
-        <v>98</v>
-      </c>
-      <c r="D8" s="3">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="3">
-        <v>109</v>
-      </c>
-      <c r="C9" s="3">
-        <v>136</v>
-      </c>
-      <c r="D9" s="3">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="3">
-        <v>424</v>
-      </c>
-      <c r="C10" s="3">
-        <v>571</v>
-      </c>
-      <c r="D10" s="3">
-        <v>9</v>
-      </c>
-      <c r="E10" s="3">
-        <v>1004</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="3">
-        <v>776</v>
-      </c>
-      <c r="C11" s="3">
-        <v>1159</v>
-      </c>
-      <c r="D11" s="3">
-        <v>9</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1944</v>
+      <c r="C12" s="4">
+        <v>546</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>549</v>
       </c>
     </row>
   </sheetData>
@@ -1469,190 +1750,190 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="A2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="4">
         <v>50</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>142000</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="4">
         <v>7090000</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="4">
         <v>11509</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="4">
         <v>616</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>37</v>
+      <c r="I2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="A3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="4">
         <v>50</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>227200</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="4">
         <v>11360000</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="4">
         <v>8513</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="4">
         <v>1335</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>43</v>
+      <c r="I3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="3">
+      <c r="A4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="3">
+      <c r="C4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="4">
+        <v>50</v>
+      </c>
+      <c r="E4" s="4">
         <v>312800</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="4">
         <v>15640000</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="4">
         <v>7689</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="4">
         <v>2034</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="4">
+        <v>50</v>
+      </c>
+      <c r="E5" s="4">
+        <v>398200</v>
+      </c>
+      <c r="F5" s="4">
+        <v>19910000</v>
+      </c>
+      <c r="G5" s="4">
+        <v>7290</v>
+      </c>
+      <c r="H5" s="4">
+        <v>2731</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="3">
-        <v>50</v>
-      </c>
-      <c r="E5" s="3">
-        <v>398200</v>
-      </c>
-      <c r="F5" s="3">
-        <v>19910000</v>
-      </c>
-      <c r="G5" s="3">
-        <v>7290</v>
-      </c>
-      <c r="H5" s="3">
-        <v>2731</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="3">
+        <v>60</v>
+      </c>
+      <c r="D6" s="4">
         <v>200</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="4">
         <v>54000000</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="4">
         <v>35001</v>
       </c>
     </row>
@@ -1671,91 +1952,91 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="4">
+        <v>11509</v>
+      </c>
+      <c r="D2" s="4">
+        <v>11509</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="4">
+        <v>8513</v>
+      </c>
+      <c r="D3" s="4">
+        <v>20022</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="4">
+        <v>7689</v>
+      </c>
+      <c r="D4" s="4">
+        <v>27711</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="3">
-        <v>11509</v>
-      </c>
-      <c r="D2" s="3">
-        <v>11509</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="3">
-        <v>8513</v>
-      </c>
-      <c r="D3" s="3">
-        <v>20022</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="3">
-        <v>7689</v>
-      </c>
-      <c r="D4" s="3">
-        <v>27711</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="3">
+      <c r="C5" s="4">
         <v>7290</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="4">
         <v>35001</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="3">
-        <v>3576</v>
+        <v>64</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2493</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="3">
-        <v>277.7</v>
+      <c r="A8" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="4">
+        <v>78.40000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1774,272 +2055,272 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="3">
+      <c r="A2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="4">
         <v>8500</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D2" s="3">
-        <v>277.7</v>
-      </c>
-      <c r="E2" s="3">
-        <v>17.7</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H2" s="5">
-        <v>10</v>
+      <c r="C2" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="4">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="E2" s="4">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H2" s="6">
+        <v>-56</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B3" s="3">
+      <c r="A3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="4">
         <v>8500</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="4">
         <v>230.2</v>
       </c>
-      <c r="E3" s="3">
-        <v>21.4</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="E3" s="4">
+        <v>26.1</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" s="6">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H3" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
         <v>8500</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="4">
+        <v>193.8</v>
+      </c>
+      <c r="E4" s="4">
+        <v>31</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H4" s="6">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="4">
+        <v>11509</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="3">
-        <v>158.8</v>
-      </c>
-      <c r="E4" s="3">
-        <v>31</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H4" s="4">
-        <v>-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5" s="3">
+      <c r="D5" s="4">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="E5" s="4">
+        <v>115</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="6">
+        <v>-73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="4">
         <v>11509</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D5" s="3">
-        <v>277.7</v>
-      </c>
-      <c r="E5" s="3">
-        <v>28.6</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" s="5">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B6" s="3">
+      <c r="D6" s="4">
+        <v>230.2</v>
+      </c>
+      <c r="E6" s="4">
+        <v>39.2</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="4">
         <v>11509</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="3">
+      <c r="C7" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="4">
+        <v>193.8</v>
+      </c>
+      <c r="E7" s="4">
+        <v>46.5</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" s="6">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="4">
+        <v>35001</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="4">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="E8" s="4">
+        <v>414.6</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" s="6">
+        <v>-223</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="4">
+        <v>35001</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="4">
         <v>230.2</v>
       </c>
-      <c r="E6" s="3">
-        <v>34.5</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" s="5">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B7" s="3">
-        <v>11509</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7" s="3">
-        <v>158.8</v>
-      </c>
-      <c r="E7" s="3">
-        <v>49.9</v>
-      </c>
-      <c r="F7" s="2" t="s">
+      <c r="E9" s="4">
+        <v>141.2</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H9" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="4">
+        <v>35001</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H7" s="4">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B8" s="3">
-        <v>35001</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D8" s="3">
-        <v>277.7</v>
-      </c>
-      <c r="E8" s="3">
-        <v>113.2</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" s="5">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B9" s="3">
-        <v>35001</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D9" s="3">
-        <v>230.2</v>
-      </c>
-      <c r="E9" s="3">
-        <v>136.5</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" s="5">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="3">
-        <v>35001</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D10" s="3">
-        <v>158.8</v>
-      </c>
-      <c r="E10" s="3">
-        <v>197.8</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H10" s="5">
-        <v>1</v>
+      <c r="D10" s="4">
+        <v>193.8</v>
+      </c>
+      <c r="E10" s="4">
+        <v>167.8</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H10" s="7">
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="6" t="s">
-        <v>85</v>
+      <c r="A12" s="8" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="6" t="s">
-        <v>86</v>
+      <c r="A13" s="8" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2053,8 +2334,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="28" spans="2:2">
-      <c r="B28" s="6" t="s">
-        <v>87</v>
+      <c r="B28" s="8" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>